<commit_message>
Add 2026 retail fuel prices (Jan-May)
</commit_message>
<xml_diff>
--- a/data/Fuel.xlsx
+++ b/data/Fuel.xlsx
@@ -20,8 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -61,13 +62,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -10598,7 +10600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1204"/>
+  <dimension ref="A1:D1218"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32272,6 +32274,258 @@
         </is>
       </c>
       <c r="D1204" t="inlineStr">
+        <is>
+          <t>Diesel</t>
+        </is>
+      </c>
+    </row>
+    <row r="1205">
+      <c r="A1205" s="4" t="n">
+        <v>46023</v>
+      </c>
+      <c r="B1205" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="C1205" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="D1205" t="inlineStr">
+        <is>
+          <t>Jet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" s="4" t="n">
+        <v>46023</v>
+      </c>
+      <c r="B1206" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="C1206" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="D1206" t="inlineStr">
+        <is>
+          <t>Diesel</t>
+        </is>
+      </c>
+    </row>
+    <row r="1207">
+      <c r="A1207" s="4" t="n">
+        <v>46054</v>
+      </c>
+      <c r="B1207" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="C1207" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="D1207" t="inlineStr">
+        <is>
+          <t>Petrol</t>
+        </is>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" s="4" t="n">
+        <v>46054</v>
+      </c>
+      <c r="B1208" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="C1208" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="D1208" t="inlineStr">
+        <is>
+          <t>Jet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1209">
+      <c r="A1209" s="4" t="n">
+        <v>46054</v>
+      </c>
+      <c r="B1209" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="C1209" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="D1209" t="inlineStr">
+        <is>
+          <t>Diesel</t>
+        </is>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" s="4" t="n">
+        <v>46082</v>
+      </c>
+      <c r="B1210" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="C1210" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="D1210" t="inlineStr">
+        <is>
+          <t>Petrol</t>
+        </is>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" s="4" t="n">
+        <v>46082</v>
+      </c>
+      <c r="B1211" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="C1211" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="D1211" t="inlineStr">
+        <is>
+          <t>Jet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" s="4" t="n">
+        <v>46082</v>
+      </c>
+      <c r="B1212" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="C1212" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="D1212" t="inlineStr">
+        <is>
+          <t>Diesel</t>
+        </is>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" s="4" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B1213" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="C1213" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="D1213" t="inlineStr">
+        <is>
+          <t>Petrol</t>
+        </is>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" s="4" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B1214" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="C1214" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="D1214" t="inlineStr">
+        <is>
+          <t>Jet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" s="4" t="n">
+        <v>46113</v>
+      </c>
+      <c r="B1215" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="C1215" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="D1215" t="inlineStr">
+        <is>
+          <t>Diesel</t>
+        </is>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" s="4" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1216" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="C1216" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="D1216" t="inlineStr">
+        <is>
+          <t>Petrol</t>
+        </is>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" s="4" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1217" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="C1217" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="D1217" t="inlineStr">
+        <is>
+          <t>Jet</t>
+        </is>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" s="4" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B1218" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="C1218" t="inlineStr">
+        <is>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="D1218" t="inlineStr">
         <is>
           <t>Diesel</t>
         </is>

</xml_diff>